<commit_message>
Creacion de catalogos de bloques unicos en clases y examenes
</commit_message>
<xml_diff>
--- a/catalogos/catalogo_bloques.xlsx
+++ b/catalogos/catalogo_bloques.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="CATALOGO_BLOQUES" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="RESUMEN" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,580 +414,1036 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B49"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>ID_BLOQUE</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>BLOQUE</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>REFERENCIA</t>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>REFERENCIAS</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>LATITUD</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>LONGITUD</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>10B</t>
+          <t>3D</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>UBEP (UNIDAD DE BIENESTAR POLITÉCNICO) / DEPORTES</t>
-        </is>
-      </c>
+          <t>3D</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>GOBIERNO FCV (FACULTAD DE CIENCIAS DE LA VIDA)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>11A</t>
+          <t>3E</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>GOBIERNO FIEC (FACULTAD DE INGENIERÍA ELÉCTRICA Y COMPUTACIÓN)</t>
-        </is>
-      </c>
+          <t>3E</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>GOBIERNO FCV (FACULTAD DE CIENCIAS DE LA VIDA)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>11B</t>
+          <t>3H</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>GOBIERNO FIEC (FACULTAD DE INGENIERÍA ELÉCTRICA Y COMPUTACIÓN)</t>
-        </is>
-      </c>
+          <t>3H</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>GOBIERNO FCV (FACULTAD DE CIENCIAS DE LA VIDA)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>11C</t>
+          <t>3K</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>GOBIERNO FIEC (FACULTAD DE INGENIERÍA ELÉCTRICA Y COMPUTACIÓN)</t>
-        </is>
-      </c>
+          <t>3K</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>GOBIERNO FCV (FACULTAD DE CIENCIAS DE LA VIDA)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>11D</t>
+          <t>3L</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>GOBIERNO FIEC (FACULTAD DE INGENIERÍA ELÉCTRICA Y COMPUTACIÓN)</t>
-        </is>
-      </c>
+          <t>3L</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>GOBIERNO FCV (FACULTAD DE CIENCIAS DE LA VIDA)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>11F</t>
+          <t>3M</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>GOBIERNO FIEC (FACULTAD DE INGENIERÍA ELÉCTRICA Y COMPUTACIÓN)</t>
-        </is>
-      </c>
+          <t>3M</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>GOBIERNO FCV (FACULTAD DE CIENCIAS DE LA VIDA)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>12C</t>
+          <t>5A</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>GOBIERNO FIMCP (FACULTAD DE INGENIERÍA MECÁNICA DE CIENCIAS DE LA PRODUCCIÓN) / STEM</t>
-        </is>
-      </c>
+          <t>5A</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>GOBIERNO FIMCM (FACULTAD DE INGENIERÍA MARÍTIMA Y CIENCIAS DEL MAR)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>12E</t>
+          <t>5F</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>GOBIERNO FIMCP (FACULTAD DE INGENIERÍA MECÁNICA DE CIENCIAS DE LA PRODUCCIÓN) / STEM</t>
-        </is>
-      </c>
+          <t>5F</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>GOBIERNO FIMCM (FACULTAD DE INGENIERÍA MARÍTIMA Y CIENCIAS DEL MAR)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>12G</t>
+          <t>5G</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>GOBIERNO FIMCP (FACULTAD DE INGENIERÍA MECÁNICA DE CIENCIAS DE LA PRODUCCIÓN) / STEM</t>
-        </is>
-      </c>
+          <t>5G</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>GOBIERNO FIMCM (FACULTAD DE INGENIERÍA MARÍTIMA Y CIENCIAS DEL MAR)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>12H</t>
+          <t>5K</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>GOBIERNO FIMCP (FACULTAD DE INGENIERÍA MECÁNICA DE CIENCIAS DE LA PRODUCCIÓN) / STEM</t>
-        </is>
-      </c>
+          <t>5K</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>GOBIERNO FIMCM (FACULTAD DE INGENIERÍA MARÍTIMA Y CIENCIAS DEL MAR)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>12I</t>
+          <t>7A</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>GOBIERNO FIMCP (FACULTAD DE INGENIERÍA MECÁNICA DE CIENCIAS DE LA PRODUCCIÓN) / STEM</t>
-        </is>
-      </c>
+          <t>7A</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>BIBLIOTECA CENTRAL</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>12J</t>
+          <t>7B</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>GOBIERNO FIMCP (FACULTAD DE INGENIERÍA MECÁNICA DE CIENCIAS DE LA PRODUCCIÓN) / STEM</t>
-        </is>
-      </c>
+          <t>7B</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>BIBLIOTECA CENTRAL</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>12K</t>
+          <t>8B</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>GOBIERNO FIMCP (FACULTAD DE INGENIERÍA MECÁNICA DE CIENCIAS DE LA PRODUCCIÓN) / STEM</t>
-        </is>
-      </c>
+          <t>8B</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>FCNM/FCSH/BCBG</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>13B</t>
+          <t>8E</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>GOBIERNO FICT (FACULTAD DE INGENIERÍA DE CIENCIAS DE LA TIERRA)</t>
-        </is>
-      </c>
+          <t>8E</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>FCNM/FCSH/BCBG</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>13C</t>
+          <t>8F</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>GOBIERNO FICT (FACULTAD DE INGENIERÍA DE CIENCIAS DE LA TIERRA)</t>
-        </is>
-      </c>
+          <t>8F</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>FCNM/FCSH/BCBG</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>13D</t>
+          <t>8G</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>GOBIERNO FICT (FACULTAD DE INGENIERÍA DE CIENCIAS DE LA TIERRA)</t>
-        </is>
-      </c>
+          <t>8G</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>FCNM/FCSH/BCBG</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>13F</t>
+          <t>8H</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>GOBIERNO FICT (FACULTAD DE INGENIERÍA DE CIENCIAS DE LA TIERRA)</t>
-        </is>
-      </c>
+          <t>8H</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>FCNM/FCSH/BCBG</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>13G</t>
+          <t>8K</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>GOBIERNO FICT (FACULTAD DE INGENIERÍA DE CIENCIAS DE LA TIERRA)</t>
-        </is>
-      </c>
+          <t>8K</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>FCNM/FCSH/BCBG</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>13H</t>
+          <t>9B</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>GOBIERNO FICT (FACULTAD DE INGENIERÍA DE CIENCIAS DE LA TIERRA)</t>
-        </is>
-      </c>
+          <t>9B</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>GOBIERNO FCSH (FACULTAD DE CIENCIAS SOCIALES Y HUMANÍSTICAS)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>14B</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr"/>
+          <t>9C</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>9C</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>GOBIERNO FCSH (FACULTAD DE CIENCIAS SOCIALES Y HUMANÍSTICAS)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>3D</t>
+          <t>9F</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>GOBIERNO FCV (FACULTAD DE CIENCIAS DE LA VIDA)</t>
-        </is>
-      </c>
+          <t>9F</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>GOBIERNO FCSH (FACULTAD DE CIENCIAS SOCIALES Y HUMANÍSTICAS)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>3E</t>
+          <t>9G</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>GOBIERNO FCV (FACULTAD DE CIENCIAS DE LA VIDA)</t>
-        </is>
-      </c>
+          <t>9G</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>GOBIERNO FCSH (FACULTAD DE CIENCIAS SOCIALES Y HUMANÍSTICAS)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>3H</t>
+          <t>9H</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>GOBIERNO FCV (FACULTAD DE CIENCIAS DE LA VIDA)</t>
-        </is>
-      </c>
+          <t>9H</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>GOBIERNO FCSH (FACULTAD DE CIENCIAS SOCIALES Y HUMANÍSTICAS)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>3K</t>
+          <t>9I</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>GOBIERNO FCV (FACULTAD DE CIENCIAS DE LA VIDA)</t>
-        </is>
-      </c>
+          <t>9I</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>GOBIERNO FCSH (FACULTAD DE CIENCIAS SOCIALES Y HUMANÍSTICAS)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>3L</t>
+          <t>9L</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>GOBIERNO FCV (FACULTAD DE CIENCIAS DE LA VIDA)</t>
-        </is>
-      </c>
+          <t>9L</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>GOBIERNO FCSH (FACULTAD DE CIENCIAS SOCIALES Y HUMANÍSTICAS)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>3M</t>
+          <t>9M</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>GOBIERNO FCV (FACULTAD DE CIENCIAS DE LA VIDA)</t>
-        </is>
-      </c>
+          <t>9M</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>GOBIERNO FCSH (FACULTAD DE CIENCIAS SOCIALES Y HUMANÍSTICAS)</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>5A</t>
+          <t>10B</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>GOBIERNO FIMCM (FACULTAD DE INGENIERÍA MARÍTIMA Y CIENCIAS DEL MAR)</t>
-        </is>
-      </c>
+          <t>10B</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>UBEP (UNIDAD DE BIENESTAR POLITÉCNICO) / DEPORTES</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>5F</t>
+          <t>11A</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>GOBIERNO FIMCM (FACULTAD DE INGENIERÍA MARÍTIMA Y CIENCIAS DEL MAR)</t>
-        </is>
-      </c>
+          <t>11A</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>GOBIERNO FIEC (FACULTAD DE INGENIERÍA ELÉCTRICA Y COMPUTACIÓN)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>5G</t>
+          <t>11B</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>GOBIERNO FIMCM (FACULTAD DE INGENIERÍA MARÍTIMA Y CIENCIAS DEL MAR)</t>
-        </is>
-      </c>
+          <t>11B</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>GOBIERNO FIEC (FACULTAD DE INGENIERÍA ELÉCTRICA Y COMPUTACIÓN)</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>5K</t>
+          <t>11C</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>GOBIERNO FIMCM (FACULTAD DE INGENIERÍA MARÍTIMA Y CIENCIAS DEL MAR)</t>
-        </is>
-      </c>
+          <t>11C</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>GOBIERNO FIEC (FACULTAD DE INGENIERÍA ELÉCTRICA Y COMPUTACIÓN)</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>7A</t>
+          <t>11D</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>BIBLIOTECA CENTRAL</t>
-        </is>
-      </c>
+          <t>11D</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>GOBIERNO FIEC (FACULTAD DE INGENIERÍA ELÉCTRICA Y COMPUTACIÓN)</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>7B</t>
+          <t>11F</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>BIBLIOTECA CENTRAL</t>
-        </is>
-      </c>
+          <t>11F</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>GOBIERNO FIEC (FACULTAD DE INGENIERÍA ELÉCTRICA Y COMPUTACIÓN)</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>8E</t>
+          <t>12C</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>FCNM/FCSH/BCBG</t>
-        </is>
-      </c>
+          <t>12C</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>GOBIERNO FIMCP (FACULTAD DE INGENIERÍA MECÁNICA DE CIENCIAS DE LA PRODUCCIÓN) / STEM</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>8F</t>
+          <t>12E</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>FCNM/FCSH/BCBG</t>
-        </is>
-      </c>
+          <t>12E</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>GOBIERNO FIMCP (FACULTAD DE INGENIERÍA MECÁNICA DE CIENCIAS DE LA PRODUCCIÓN) / STEM</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>8G</t>
+          <t>12G</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>FCNM/FCSH/BCBG</t>
-        </is>
-      </c>
+          <t>12G</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>GOBIERNO FIMCP (FACULTAD DE INGENIERÍA MECÁNICA DE CIENCIAS DE LA PRODUCCIÓN) / STEM</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>8H</t>
+          <t>12H</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>FCNM/FCSH/BCBG</t>
-        </is>
-      </c>
+          <t>12H</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>GOBIERNO FIMCP (FACULTAD DE INGENIERÍA MECÁNICA DE CIENCIAS DE LA PRODUCCIÓN) / STEM</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>8K</t>
+          <t>12I</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>FCNM/FCSH/BCBG</t>
-        </is>
-      </c>
+          <t>12I</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>GOBIERNO FIMCP (FACULTAD DE INGENIERÍA MECÁNICA DE CIENCIAS DE LA PRODUCCIÓN) / STEM</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>9B</t>
+          <t>12J</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>GOBIERNO FCSH (FACULTAD DE CIENCIAS SOCIALES Y HUMANÍSTICAS)</t>
-        </is>
-      </c>
+          <t>12J</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>GOBIERNO FIMCP (FACULTAD DE INGENIERÍA MECÁNICA DE CIENCIAS DE LA PRODUCCIÓN) / STEM</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>9C</t>
+          <t>12K</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>GOBIERNO FCSH (FACULTAD DE CIENCIAS SOCIALES Y HUMANÍSTICAS)</t>
-        </is>
-      </c>
+          <t>12K</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>GOBIERNO FIMCP (FACULTAD DE INGENIERÍA MECÁNICA DE CIENCIAS DE LA PRODUCCIÓN) / STEM</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>9F</t>
+          <t>13B</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>GOBIERNO FCSH (FACULTAD DE CIENCIAS SOCIALES Y HUMANÍSTICAS)</t>
-        </is>
-      </c>
+          <t>13B</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>GOBIERNO FICT (FACULTAD DE INGENIERÍA DE CIENCIAS DE LA TIERRA)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>9G</t>
+          <t>13C</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>GOBIERNO FCSH (FACULTAD DE CIENCIAS SOCIALES Y HUMANÍSTICAS)</t>
-        </is>
-      </c>
+          <t>13C</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>GOBIERNO FICT (FACULTAD DE INGENIERÍA DE CIENCIAS DE LA TIERRA)</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>9H</t>
+          <t>13D</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>GOBIERNO FCSH (FACULTAD DE CIENCIAS SOCIALES Y HUMANÍSTICAS)</t>
-        </is>
-      </c>
+          <t>13D</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>GOBIERNO FICT (FACULTAD DE INGENIERÍA DE CIENCIAS DE LA TIERRA)</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>9I</t>
+          <t>13F</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>GOBIERNO FCSH (FACULTAD DE CIENCIAS SOCIALES Y HUMANÍSTICAS)</t>
-        </is>
-      </c>
+          <t>13F</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>GOBIERNO FICT (FACULTAD DE INGENIERÍA DE CIENCIAS DE LA TIERRA)</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>9L</t>
+          <t>13G</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>GOBIERNO FCSH (FACULTAD DE CIENCIAS SOCIALES Y HUMANÍSTICAS)</t>
-        </is>
-      </c>
+          <t>13G</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>GOBIERNO FICT (FACULTAD DE INGENIERÍA DE CIENCIAS DE LA TIERRA)</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>9M</t>
+          <t>13H</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>GOBIERNO FCSH (FACULTAD DE CIENCIAS SOCIALES Y HUMANÍSTICAS)</t>
-        </is>
-      </c>
+          <t>13H</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>GOBIERNO FICT (FACULTAD DE INGENIERÍA DE CIENCIAS DE LA TIERRA)</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>AULAS EDCOM</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr"/>
+          <t>14B</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>14B</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>DEPORTES</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr"/>
+          <t>AULAS EDCOM</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>AULAS EDCOM</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
+          <t>DEPORTES</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>DEPORTES</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
           <t>GEA</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr"/>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>GEA</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>METRICA</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>CANTIDAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>BLOQUES UNICOS</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BLOQUES EN CLASES</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>BLOQUES EN EXAMENES</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BLOQUES EN AMBAS FUENTES</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>COORDENADAS COMPLETAS</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>COORDENADAS PENDIENTES</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>49</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Limpiezas completadas, heatmaps creados y catalogos de bloques modificados
</commit_message>
<xml_diff>
--- a/catalogos/catalogo_bloques.xlsx
+++ b/catalogos/catalogo_bloques.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carla\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A8CE208-181C-4E98-90C5-5CF16E67E601}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56BE4B55-6A60-48B0-819F-C3805FC1D8C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="82">
   <si>
     <t>ID_BLOQUE</t>
   </si>
@@ -32,6 +32,9 @@
     <t>REFERENCIAS</t>
   </si>
   <si>
+    <t>FACULTAD</t>
+  </si>
+  <si>
     <t>LATITUD</t>
   </si>
   <si>
@@ -234,6 +237,36 @@
   </si>
   <si>
     <t>COORDENADAS PENDIENTES</t>
+  </si>
+  <si>
+    <t>FCV</t>
+  </si>
+  <si>
+    <t>FIMCM</t>
+  </si>
+  <si>
+    <t>FCSH</t>
+  </si>
+  <si>
+    <t>FCNM</t>
+  </si>
+  <si>
+    <t>UBEP</t>
+  </si>
+  <si>
+    <t>FIEC</t>
+  </si>
+  <si>
+    <t>FICT</t>
+  </si>
+  <si>
+    <t>FIMCP</t>
+  </si>
+  <si>
+    <t>FADCOM</t>
+  </si>
+  <si>
+    <t>COLISEO</t>
   </si>
 </sst>
 </file>
@@ -573,13 +606,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:F50"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="3" max="3" width="84.21875" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -595,825 +625,987 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E2">
         <v>-2.1506130458069799</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <v>-79.957712891260996</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
         <v>7</v>
       </c>
-      <c r="B3" t="s">
+      <c r="D3" t="s">
+        <v>72</v>
+      </c>
+      <c r="E3">
+        <v>-2.1504655372333898</v>
+      </c>
+      <c r="F3">
+        <v>-79.957417666181996</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" t="s">
         <v>7</v>
       </c>
-      <c r="C3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3">
-        <v>-2.1504655372333898</v>
-      </c>
-      <c r="E3">
-        <v>-79.957417666181996</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4">
+      <c r="D4" t="s">
+        <v>72</v>
+      </c>
+      <c r="E4">
         <v>-2.1522218533900102</v>
       </c>
-      <c r="E4">
+      <c r="F4">
         <v>-79.955962234068707</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5">
+        <v>7</v>
+      </c>
+      <c r="D5" t="s">
+        <v>72</v>
+      </c>
+      <c r="E5">
         <v>-2.1512651162640002</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <v>-79.954164671961394</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C6" t="s">
-        <v>6</v>
-      </c>
-      <c r="D6">
+        <v>7</v>
+      </c>
+      <c r="D6" t="s">
+        <v>72</v>
+      </c>
+      <c r="E6">
         <v>-2.1515615118301499</v>
       </c>
-      <c r="E6">
+      <c r="F6">
         <v>-79.954330218745596</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D7">
+        <v>7</v>
+      </c>
+      <c r="D7" t="s">
+        <v>72</v>
+      </c>
+      <c r="E7">
         <v>-2.15188410043447</v>
       </c>
-      <c r="E7">
+      <c r="F7">
         <v>-79.953981190942997</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C8" t="s">
-        <v>13</v>
-      </c>
-      <c r="D8">
+        <v>14</v>
+      </c>
+      <c r="D8" t="s">
+        <v>73</v>
+      </c>
+      <c r="E8">
         <v>-2.14692893015954</v>
       </c>
-      <c r="E8">
+      <c r="F8">
         <v>-79.962765702698903</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" t="s">
         <v>14</v>
       </c>
-      <c r="B9" t="s">
+      <c r="D9" t="s">
+        <v>73</v>
+      </c>
+      <c r="E9">
+        <v>-2.1462818685073901</v>
+      </c>
+      <c r="F9">
+        <v>-79.962437226268804</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" t="s">
         <v>14</v>
       </c>
-      <c r="C9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D9">
-        <v>-2.1462818685073901</v>
-      </c>
-      <c r="E9">
-        <v>-79.962437226268804</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" t="s">
-        <v>15</v>
-      </c>
-      <c r="C10" t="s">
-        <v>13</v>
-      </c>
-      <c r="D10">
+      <c r="D10" t="s">
+        <v>73</v>
+      </c>
+      <c r="E10">
         <v>-2.1464485793034598</v>
       </c>
-      <c r="E10">
+      <c r="F10">
         <v>-79.962456958595396</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C11" t="s">
-        <v>13</v>
-      </c>
-      <c r="D11">
+        <v>14</v>
+      </c>
+      <c r="D11" t="s">
+        <v>73</v>
+      </c>
+      <c r="E11">
         <v>-2.1467846897301701</v>
       </c>
-      <c r="E11">
+      <c r="F11">
         <v>-79.963186157719207</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D12">
+        <v>19</v>
+      </c>
+      <c r="D12" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12">
         <v>-2.14753270978176</v>
       </c>
-      <c r="E12">
+      <c r="F12">
         <v>-79.966290890950106</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" t="s">
         <v>19</v>
       </c>
-      <c r="B13" t="s">
+      <c r="D13" t="s">
         <v>19</v>
       </c>
-      <c r="C13" t="s">
-        <v>18</v>
-      </c>
-      <c r="D13">
+      <c r="E13">
         <v>-2.14708777573775</v>
       </c>
-      <c r="E13">
+      <c r="F13">
         <v>-79.966009258999193</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C14" t="s">
-        <v>21</v>
-      </c>
-      <c r="D14">
+        <v>22</v>
+      </c>
+      <c r="D14" t="s">
+        <v>74</v>
+      </c>
+      <c r="E14">
         <v>-2.1482025739853898</v>
       </c>
-      <c r="E14">
+      <c r="F14">
         <v>-79.968706875818796</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" t="s">
+        <v>23</v>
+      </c>
+      <c r="C15" t="s">
         <v>22</v>
       </c>
-      <c r="B15" t="s">
+      <c r="D15" t="s">
+        <v>74</v>
+      </c>
+      <c r="E15">
+        <v>-2.1488115020934799</v>
+      </c>
+      <c r="F15">
+        <v>-79.967901091480101</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" t="s">
         <v>22</v>
       </c>
-      <c r="C15" t="s">
-        <v>21</v>
-      </c>
-      <c r="D15">
-        <v>-2.1488115020934799</v>
-      </c>
-      <c r="E15">
-        <v>-79.967901091480101</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>23</v>
-      </c>
-      <c r="B16" t="s">
-        <v>23</v>
-      </c>
-      <c r="C16" t="s">
-        <v>21</v>
-      </c>
-      <c r="D16">
+      <c r="D16" t="s">
+        <v>74</v>
+      </c>
+      <c r="E16">
         <v>-2.14877783195857</v>
       </c>
-      <c r="E16">
+      <c r="F16">
         <v>-79.967604299026306</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B17" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C17" t="s">
-        <v>21</v>
-      </c>
-      <c r="D17">
+        <v>22</v>
+      </c>
+      <c r="D17" t="s">
+        <v>74</v>
+      </c>
+      <c r="E17">
         <v>-2.14862882368775</v>
       </c>
-      <c r="E17">
+      <c r="F17">
         <v>-79.967277397200903</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B18" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C18" t="s">
-        <v>21</v>
-      </c>
-      <c r="D18">
+        <v>22</v>
+      </c>
+      <c r="D18" t="s">
+        <v>74</v>
+      </c>
+      <c r="E18">
         <v>-2.1484359125469998</v>
       </c>
-      <c r="E18">
+      <c r="F18">
         <v>-79.967436718680901</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C19" t="s">
-        <v>21</v>
-      </c>
-      <c r="D19">
+        <v>22</v>
+      </c>
+      <c r="D19" t="s">
+        <v>74</v>
+      </c>
+      <c r="E19">
         <v>-2.1451807327959802</v>
       </c>
-      <c r="E19">
+      <c r="F19">
         <v>-79.969324733767195</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B20" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C20" t="s">
-        <v>28</v>
-      </c>
-      <c r="D20">
+        <v>29</v>
+      </c>
+      <c r="D20" t="s">
+        <v>75</v>
+      </c>
+      <c r="E20">
         <v>-2.1471559372114499</v>
       </c>
-      <c r="E20">
+      <c r="F20">
         <v>-79.967232783236895</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
+        <v>30</v>
+      </c>
+      <c r="B21" t="s">
+        <v>30</v>
+      </c>
+      <c r="C21" t="s">
         <v>29</v>
       </c>
-      <c r="B21" t="s">
+      <c r="D21" t="s">
+        <v>75</v>
+      </c>
+      <c r="E21">
+        <v>-2.1472363469825901</v>
+      </c>
+      <c r="F21">
+        <v>-79.967087273393204</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>31</v>
+      </c>
+      <c r="B22" t="s">
+        <v>31</v>
+      </c>
+      <c r="C22" t="s">
         <v>29</v>
       </c>
-      <c r="C21" t="s">
-        <v>28</v>
-      </c>
-      <c r="D21">
-        <v>-2.1472363469825901</v>
-      </c>
-      <c r="E21">
-        <v>-79.967087273393204</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>30</v>
-      </c>
-      <c r="B22" t="s">
-        <v>30</v>
-      </c>
-      <c r="C22" t="s">
-        <v>28</v>
-      </c>
-      <c r="D22">
+      <c r="D22" t="s">
+        <v>75</v>
+      </c>
+      <c r="E22">
         <v>-2.14713047411627</v>
       </c>
-      <c r="E22">
+      <c r="F22">
         <v>-79.967838291925602</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B23" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C23" t="s">
-        <v>28</v>
-      </c>
-      <c r="D23">
+        <v>29</v>
+      </c>
+      <c r="D23" t="s">
+        <v>75</v>
+      </c>
+      <c r="E23">
         <v>-2.1467106916843202</v>
       </c>
-      <c r="E23">
+      <c r="F23">
         <v>-79.967567934955596</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B24" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C24" t="s">
-        <v>28</v>
-      </c>
-      <c r="D24">
+        <v>29</v>
+      </c>
+      <c r="D24" t="s">
+        <v>75</v>
+      </c>
+      <c r="E24">
         <v>-2.1465655953296001</v>
       </c>
-      <c r="E24">
+      <c r="F24">
         <v>-79.967992518943205</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B25" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C25" t="s">
-        <v>28</v>
-      </c>
-      <c r="D25">
+        <v>29</v>
+      </c>
+      <c r="D25" t="s">
+        <v>75</v>
+      </c>
+      <c r="E25">
         <v>-2.14605406680508</v>
       </c>
-      <c r="E25">
+      <c r="F25">
         <v>-79.967226882198801</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B26" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C26" t="s">
-        <v>28</v>
-      </c>
-      <c r="D26">
+        <v>29</v>
+      </c>
+      <c r="D26" t="s">
+        <v>75</v>
+      </c>
+      <c r="E26">
         <v>-2.14657211976755</v>
       </c>
-      <c r="E26">
+      <c r="F26">
         <v>-79.967165663835004</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B27" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C27" t="s">
-        <v>28</v>
-      </c>
-      <c r="D27">
+        <v>29</v>
+      </c>
+      <c r="D27" t="s">
+        <v>75</v>
+      </c>
+      <c r="E27">
         <v>-2.1468414320470401</v>
       </c>
-      <c r="E27">
+      <c r="F27">
         <v>-79.966619432882894</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B28" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C28" t="s">
-        <v>37</v>
-      </c>
-      <c r="D28">
+        <v>38</v>
+      </c>
+      <c r="D28" t="s">
+        <v>76</v>
+      </c>
+      <c r="E28">
         <v>-2.1431651136910901</v>
       </c>
-      <c r="E28">
+      <c r="F28">
         <v>-79.965978413585205</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C29" t="s">
-        <v>39</v>
-      </c>
-      <c r="D29">
+        <v>40</v>
+      </c>
+      <c r="D29" t="s">
+        <v>77</v>
+      </c>
+      <c r="E29">
         <v>-2.1445551724890901</v>
       </c>
-      <c r="E29">
+      <c r="F29">
         <v>-79.967680647969402</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
+        <v>41</v>
+      </c>
+      <c r="B30" t="s">
+        <v>41</v>
+      </c>
+      <c r="C30" t="s">
         <v>40</v>
       </c>
-      <c r="B30" t="s">
+      <c r="D30" t="s">
+        <v>77</v>
+      </c>
+      <c r="E30">
+        <v>-2.1450604146821801</v>
+      </c>
+      <c r="F30">
+        <v>-79.967361465101703</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>42</v>
+      </c>
+      <c r="B31" t="s">
+        <v>42</v>
+      </c>
+      <c r="C31" t="s">
         <v>40</v>
       </c>
-      <c r="C30" t="s">
-        <v>39</v>
-      </c>
-      <c r="D30">
-        <v>-2.1450604146821801</v>
-      </c>
-      <c r="E30">
-        <v>-79.967361465101703</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>41</v>
-      </c>
-      <c r="B31" t="s">
-        <v>41</v>
-      </c>
-      <c r="C31" t="s">
-        <v>39</v>
-      </c>
-      <c r="D31">
+      <c r="D31" t="s">
+        <v>77</v>
+      </c>
+      <c r="E31">
         <v>-2.14577933318269</v>
       </c>
-      <c r="E31">
+      <c r="F31">
         <v>-79.966801752073195</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B32" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C32" t="s">
-        <v>39</v>
-      </c>
-      <c r="D32">
+        <v>40</v>
+      </c>
+      <c r="D32" t="s">
+        <v>77</v>
+      </c>
+      <c r="E32">
         <v>-2.1454691648712299</v>
       </c>
-      <c r="E32">
+      <c r="F32">
         <v>-79.966179952014599</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B33" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C33" t="s">
-        <v>39</v>
-      </c>
-      <c r="D33">
+        <v>40</v>
+      </c>
+      <c r="D33" t="s">
+        <v>77</v>
+      </c>
+      <c r="E33">
         <v>-2.1450681488067702</v>
       </c>
-      <c r="E33">
+      <c r="F33">
         <v>-79.9665792284178</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B34" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C34" t="s">
-        <v>45</v>
-      </c>
-      <c r="D34">
+        <v>46</v>
+      </c>
+      <c r="D34" t="s">
+        <v>79</v>
+      </c>
+      <c r="E34">
         <v>-2.1450134888592798</v>
       </c>
-      <c r="E34">
+      <c r="F34">
         <v>-79.965849254576895</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
+        <v>47</v>
+      </c>
+      <c r="B35" t="s">
+        <v>47</v>
+      </c>
+      <c r="C35" t="s">
         <v>46</v>
       </c>
-      <c r="B35" t="s">
+      <c r="D35" t="s">
+        <v>79</v>
+      </c>
+      <c r="E35">
+        <v>-2.1446205055376901</v>
+      </c>
+      <c r="F35">
+        <v>-79.966324456030605</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>48</v>
+      </c>
+      <c r="B36" t="s">
+        <v>48</v>
+      </c>
+      <c r="C36" t="s">
         <v>46</v>
       </c>
-      <c r="C35" t="s">
-        <v>45</v>
-      </c>
-      <c r="D35">
-        <v>-2.1446205055376901</v>
-      </c>
-      <c r="E35">
-        <v>-79.966324456030605</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A36" t="s">
-        <v>47</v>
-      </c>
-      <c r="B36" t="s">
-        <v>47</v>
-      </c>
-      <c r="C36" t="s">
-        <v>45</v>
-      </c>
-      <c r="D36">
+      <c r="D36" t="s">
+        <v>79</v>
+      </c>
+      <c r="E36">
         <v>-2.1444697369554402</v>
       </c>
-      <c r="E36">
+      <c r="F36">
         <v>-79.966386817392205</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B37" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C37" t="s">
-        <v>45</v>
-      </c>
-      <c r="D37">
+        <v>46</v>
+      </c>
+      <c r="D37" t="s">
+        <v>79</v>
+      </c>
+      <c r="E37">
         <v>-2.1442352080145302</v>
       </c>
-      <c r="E37">
+      <c r="F37">
         <v>-79.966318421062695</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B38" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C38" t="s">
-        <v>45</v>
-      </c>
-      <c r="D38">
+        <v>46</v>
+      </c>
+      <c r="D38" t="s">
+        <v>79</v>
+      </c>
+      <c r="E38">
         <v>-2.14406979633636</v>
       </c>
-      <c r="E38">
+      <c r="F38">
         <v>-79.965983636150895</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B39" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C39" t="s">
-        <v>45</v>
-      </c>
-      <c r="D39">
+        <v>46</v>
+      </c>
+      <c r="D39" t="s">
+        <v>79</v>
+      </c>
+      <c r="E39">
         <v>-2.14408051766106</v>
       </c>
-      <c r="E39">
+      <c r="F39">
         <v>-79.966225705522206</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B40" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C40" t="s">
-        <v>45</v>
-      </c>
-      <c r="D40">
+        <v>46</v>
+      </c>
+      <c r="D40" t="s">
+        <v>79</v>
+      </c>
+      <c r="E40">
         <v>-2.1439076362876501</v>
       </c>
-      <c r="E40">
+      <c r="F40">
         <v>-79.966406084080603</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B41" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C41" t="s">
-        <v>53</v>
-      </c>
-      <c r="D41">
+        <v>54</v>
+      </c>
+      <c r="D41" t="s">
+        <v>78</v>
+      </c>
+      <c r="E41">
         <v>-2.1455764124913901</v>
       </c>
-      <c r="E41">
+      <c r="F41">
         <v>-79.965043753456698</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
+        <v>55</v>
+      </c>
+      <c r="B42" t="s">
+        <v>55</v>
+      </c>
+      <c r="C42" t="s">
         <v>54</v>
       </c>
-      <c r="B42" t="s">
+      <c r="D42" t="s">
+        <v>78</v>
+      </c>
+      <c r="E42">
+        <v>-2.1453341250232101</v>
+      </c>
+      <c r="F42">
+        <v>-79.964774648158297</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>56</v>
+      </c>
+      <c r="B43" t="s">
+        <v>56</v>
+      </c>
+      <c r="C43" t="s">
         <v>54</v>
       </c>
-      <c r="C42" t="s">
-        <v>53</v>
-      </c>
-      <c r="D42">
-        <v>-2.1453341250232101</v>
-      </c>
-      <c r="E42">
-        <v>-79.964774648158297</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A43" t="s">
-        <v>55</v>
-      </c>
-      <c r="B43" t="s">
-        <v>55</v>
-      </c>
-      <c r="C43" t="s">
-        <v>53</v>
-      </c>
-      <c r="D43">
+      <c r="D43" t="s">
+        <v>78</v>
+      </c>
+      <c r="E43">
         <v>-2.1455106480481398</v>
       </c>
-      <c r="E43">
+      <c r="F43">
         <v>-79.964787226490003</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B44" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C44" t="s">
-        <v>53</v>
-      </c>
-      <c r="D44">
+        <v>54</v>
+      </c>
+      <c r="D44" t="s">
+        <v>78</v>
+      </c>
+      <c r="E44">
         <v>-2.1459508671274001</v>
       </c>
-      <c r="E44">
+      <c r="F44">
         <v>-79.965133739351799</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B45" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C45" t="s">
-        <v>53</v>
-      </c>
-      <c r="D45">
+        <v>54</v>
+      </c>
+      <c r="D45" t="s">
+        <v>78</v>
+      </c>
+      <c r="E45">
         <v>-2.1459106031912301</v>
       </c>
-      <c r="E45">
+      <c r="F45">
         <v>-79.965488310645398</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B46" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C46" t="s">
-        <v>53</v>
-      </c>
-      <c r="D46">
+        <v>54</v>
+      </c>
+      <c r="D46" t="s">
+        <v>78</v>
+      </c>
+      <c r="E46">
         <v>-2.14596965696169</v>
       </c>
-      <c r="E46">
+      <c r="F46">
         <v>-79.965900634094595</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B47" t="s">
-        <v>59</v>
-      </c>
-      <c r="D47">
+        <v>60</v>
+      </c>
+      <c r="C47" t="s">
+        <v>80</v>
+      </c>
+      <c r="D47" t="s">
+        <v>80</v>
+      </c>
+      <c r="E47">
         <v>-2.1436048131634502</v>
       </c>
-      <c r="E47">
+      <c r="F47">
         <v>-79.962187969643296</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B48" t="s">
-        <v>60</v>
-      </c>
-      <c r="D48">
+        <v>61</v>
+      </c>
+      <c r="C48" t="s">
+        <v>80</v>
+      </c>
+      <c r="D48" t="s">
+        <v>80</v>
+      </c>
+      <c r="E48">
         <v>-2.1440955263808901</v>
       </c>
-      <c r="E48">
+      <c r="F48">
         <v>-79.962343856210794</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B49" t="s">
-        <v>61</v>
-      </c>
-      <c r="D49">
+        <v>62</v>
+      </c>
+      <c r="C49" t="s">
+        <v>81</v>
+      </c>
+      <c r="D49" t="s">
+        <v>81</v>
+      </c>
+      <c r="E49">
         <v>-2.1451163715819499</v>
       </c>
-      <c r="E49">
+      <c r="F49">
         <v>-79.964225087995302</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B50" t="s">
-        <v>62</v>
-      </c>
-      <c r="D50">
+        <v>63</v>
+      </c>
+      <c r="C50" t="s">
+        <v>63</v>
+      </c>
+      <c r="D50" t="s">
+        <v>63</v>
+      </c>
+      <c r="E50">
         <v>-2.14012557081388</v>
       </c>
-      <c r="E50">
+      <c r="F50">
         <v>-79.962625817992304</v>
       </c>
     </row>
@@ -1429,15 +1621,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B2">
         <v>49</v>
@@ -1445,7 +1637,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B3">
         <v>48</v>
@@ -1453,7 +1645,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B4">
         <v>40</v>
@@ -1461,7 +1653,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B5">
         <v>39</v>
@@ -1469,18 +1661,18 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B6">
-        <v>0</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B7">
-        <v>49</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>